<commit_message>
Move VFD Decision Matrix out of BOM file to vfd/ folder
VFD Decision Matrix is a design-decision document, not a Bill of
Materials. Moved from BOM/BOM_Combined_As_Built.xlsx (where it was
a sheet) to its own standalone file in vfd/ alongside the other
VFD documentation:

- vfd/VFD_Decision_Matrix.xlsx (working source)
- vfd/VFD_Decision_Matrix.pdf (rendered)

The combined BOM now contains only BOM-relevant sheets: 'Combined BOM'
(as-built items) and 'Excluded - Not Used' (items considered but
not installed, with reasons).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BOM/BOM_Combined_As_Built.xlsx
+++ b/BOM/BOM_Combined_As_Built.xlsx
@@ -9,7 +9,6 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Combined BOM" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excluded - Not Used" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VFD Decision Matrix" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -507,7 +506,6 @@
       <c r="A3" t="n">
         <v>1</v>
       </c>
-      <c r="B3" t="inlineStr"/>
       <c r="C3" s="3" t="inlineStr">
         <is>
           <t>AC Motor (bench test unit)</t>
@@ -541,7 +539,6 @@
       <c r="A4" t="n">
         <v>2</v>
       </c>
-      <c r="B4" t="inlineStr"/>
       <c r="C4" s="3" t="inlineStr">
         <is>
           <t>VFD (Variable Frequency Drive)</t>
@@ -575,7 +572,6 @@
       <c r="A5" t="n">
         <v>3</v>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" s="3" t="inlineStr">
         <is>
           <t>Dynamic Braking Resistor</t>
@@ -616,7 +612,6 @@
       <c r="A7" t="n">
         <v>4</v>
       </c>
-      <c r="B7" t="inlineStr"/>
       <c r="C7" s="3" t="inlineStr">
         <is>
           <t>Main Power Switch</t>
@@ -650,7 +645,6 @@
       <c r="A8" t="n">
         <v>5</v>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" s="3" t="inlineStr">
         <is>
           <t>VFD Branch Breaker</t>
@@ -684,7 +678,6 @@
       <c r="A9" t="n">
         <v>6</v>
       </c>
-      <c r="B9" t="inlineStr"/>
       <c r="C9" s="3" t="inlineStr">
         <is>
           <t>DC Power Supply</t>
@@ -718,7 +711,6 @@
       <c r="A10" t="n">
         <v>7</v>
       </c>
-      <c r="B10" t="inlineStr"/>
       <c r="C10" s="3" t="inlineStr">
         <is>
           <t>Main Power Contactor</t>
@@ -752,7 +744,6 @@
       <c r="A11" t="n">
         <v>8</v>
       </c>
-      <c r="B11" t="inlineStr"/>
       <c r="C11" s="3" t="inlineStr">
         <is>
           <t>Fuse Block - 24V Button Common</t>
@@ -786,7 +777,6 @@
       <c r="A12" t="n">
         <v>9</v>
       </c>
-      <c r="B12" t="inlineStr"/>
       <c r="C12" s="3" t="inlineStr">
         <is>
           <t>Fuse Block - AC Branches</t>
@@ -827,7 +817,6 @@
       <c r="A14" t="n">
         <v>10</v>
       </c>
-      <c r="B14" t="inlineStr"/>
       <c r="C14" s="3" t="inlineStr">
         <is>
           <t>PLC CPU / Ethernet Module</t>
@@ -861,7 +850,6 @@
       <c r="A15" t="n">
         <v>11</v>
       </c>
-      <c r="B15" t="inlineStr"/>
       <c r="C15" s="3" t="inlineStr">
         <is>
           <t>PLC Rack / Base</t>
@@ -895,7 +883,6 @@
       <c r="A16" t="n">
         <v>12</v>
       </c>
-      <c r="B16" t="inlineStr"/>
       <c r="C16" s="3" t="inlineStr">
         <is>
           <t>Discrete Input Module (24 VDC)</t>
@@ -929,7 +916,6 @@
       <c r="A17" t="n">
         <v>13</v>
       </c>
-      <c r="B17" t="inlineStr"/>
       <c r="C17" s="3" t="inlineStr">
         <is>
           <t>Analog Current Input Module</t>
@@ -963,7 +949,6 @@
       <c r="A18" t="n">
         <v>14</v>
       </c>
-      <c r="B18" t="inlineStr"/>
       <c r="C18" s="3" t="inlineStr">
         <is>
           <t>RTD Input Module</t>
@@ -997,7 +982,6 @@
       <c r="A19" t="n">
         <v>15</v>
       </c>
-      <c r="B19" t="inlineStr"/>
       <c r="C19" s="3" t="inlineStr">
         <is>
           <t>Relay Output Module</t>
@@ -1031,7 +1015,6 @@
       <c r="A20" t="n">
         <v>16</v>
       </c>
-      <c r="B20" t="inlineStr"/>
       <c r="C20" s="3" t="inlineStr">
         <is>
           <t>Analog Voltage Output Module</t>
@@ -1065,7 +1048,6 @@
       <c r="A21" t="n">
         <v>17</v>
       </c>
-      <c r="B21" t="inlineStr"/>
       <c r="C21" s="3" t="inlineStr">
         <is>
           <t>PLC Rack Filler Panels</t>
@@ -1106,7 +1088,6 @@
       <c r="A23" t="n">
         <v>18</v>
       </c>
-      <c r="B23" t="inlineStr"/>
       <c r="C23" s="3" t="inlineStr">
         <is>
           <t>C-More Micro Touch Panel</t>
@@ -1147,7 +1128,6 @@
       <c r="A25" t="n">
         <v>19</v>
       </c>
-      <c r="B25" t="inlineStr"/>
       <c r="C25" s="3" t="inlineStr">
         <is>
           <t>Forward Pushbutton Head</t>
@@ -1181,7 +1161,6 @@
       <c r="A26" t="n">
         <v>20</v>
       </c>
-      <c r="B26" t="inlineStr"/>
       <c r="C26" s="3" t="inlineStr">
         <is>
           <t>Reverse Pushbutton Head</t>
@@ -1215,7 +1194,6 @@
       <c r="A27" t="n">
         <v>21</v>
       </c>
-      <c r="B27" t="inlineStr"/>
       <c r="C27" s="3" t="inlineStr">
         <is>
           <t>Deadman/Run Pushbutton Head</t>
@@ -1249,7 +1227,6 @@
       <c r="A28" t="n">
         <v>22</v>
       </c>
-      <c r="B28" t="inlineStr"/>
       <c r="C28" s="3" t="inlineStr">
         <is>
           <t>Reset Pushbutton Head</t>
@@ -1283,7 +1260,6 @@
       <c r="A29" t="n">
         <v>23</v>
       </c>
-      <c r="B29" t="inlineStr"/>
       <c r="C29" s="3" t="inlineStr">
         <is>
           <t>NO Contact Block (1NO finger-safe)</t>
@@ -1317,7 +1293,6 @@
       <c r="A30" t="n">
         <v>24</v>
       </c>
-      <c r="B30" t="inlineStr"/>
       <c r="C30" s="3" t="inlineStr">
         <is>
           <t>LED Block - Green (24V DC)</t>
@@ -1351,7 +1326,6 @@
       <c r="A31" t="n">
         <v>25</v>
       </c>
-      <c r="B31" t="inlineStr"/>
       <c r="C31" s="3" t="inlineStr">
         <is>
           <t>LED Block - Yellow (24V DC)</t>
@@ -1385,7 +1359,6 @@
       <c r="A32" t="n">
         <v>26</v>
       </c>
-      <c r="B32" t="inlineStr"/>
       <c r="C32" s="3" t="inlineStr">
         <is>
           <t>LED Block - Blue (24V DC)</t>
@@ -1419,7 +1392,6 @@
       <c r="A33" t="n">
         <v>27</v>
       </c>
-      <c r="B33" t="inlineStr"/>
       <c r="C33" s="3" t="inlineStr">
         <is>
           <t>LED Block - Red (24V DC)</t>
@@ -1453,7 +1425,6 @@
       <c r="A34" t="n">
         <v>28</v>
       </c>
-      <c r="B34" t="inlineStr"/>
       <c r="C34" s="3" t="inlineStr">
         <is>
           <t>Emergency Stop Pushbutton</t>
@@ -1487,7 +1458,6 @@
       <c r="A35" t="n">
         <v>29</v>
       </c>
-      <c r="B35" t="inlineStr"/>
       <c r="C35" s="3" t="inlineStr">
         <is>
           <t>Panel Indicator Light - Error/Fault</t>
@@ -1528,7 +1498,6 @@
       <c r="A37" t="n">
         <v>30</v>
       </c>
-      <c r="B37" t="inlineStr"/>
       <c r="C37" s="3" t="inlineStr">
         <is>
           <t>Banana Socket - Blue (4 mm)</t>
@@ -1562,7 +1531,6 @@
       <c r="A38" t="n">
         <v>31</v>
       </c>
-      <c r="B38" t="inlineStr"/>
       <c r="C38" s="3" t="inlineStr">
         <is>
           <t>Banana Socket - White (4 mm)</t>
@@ -1596,7 +1564,6 @@
       <c r="A39" t="n">
         <v>32</v>
       </c>
-      <c r="B39" t="inlineStr"/>
       <c r="C39" s="3" t="inlineStr">
         <is>
           <t>Banana Socket - Red (4 mm)</t>
@@ -1637,7 +1604,6 @@
       <c r="A41" t="n">
         <v>33</v>
       </c>
-      <c r="B41" t="inlineStr"/>
       <c r="C41" s="3" t="inlineStr">
         <is>
           <t>Slotted Wire Duct (Type G, 1" x 1")</t>
@@ -1671,7 +1637,6 @@
       <c r="A42" t="n">
         <v>34</v>
       </c>
-      <c r="B42" t="inlineStr"/>
       <c r="C42" s="3" t="inlineStr">
         <is>
           <t>Duct Cover for G1X1LG6</t>
@@ -1705,7 +1670,6 @@
       <c r="A43" t="n">
         <v>35</v>
       </c>
-      <c r="B43" t="inlineStr"/>
       <c r="C43" s="3" t="inlineStr">
         <is>
           <t>Insulated Crimp Ferrules, 12 AWG (gray)</t>
@@ -1739,7 +1703,6 @@
       <c r="A44" t="n">
         <v>36</v>
       </c>
-      <c r="B44" t="inlineStr"/>
       <c r="C44" s="3" t="inlineStr">
         <is>
           <t>Control Wire - 18 AWG stranded Blue</t>
@@ -1773,7 +1736,6 @@
       <c r="A45" t="n">
         <v>37</v>
       </c>
-      <c r="B45" t="inlineStr"/>
       <c r="C45" s="3" t="inlineStr">
         <is>
           <t>Return Wire - 18 AWG White or Blue/W</t>
@@ -1807,7 +1769,6 @@
       <c r="A46" t="n">
         <v>38</v>
       </c>
-      <c r="B46" t="inlineStr"/>
       <c r="C46" s="3" t="inlineStr">
         <is>
           <t>Power Wire - 12 AWG Black</t>
@@ -1841,7 +1802,6 @@
       <c r="A47" t="n">
         <v>39</v>
       </c>
-      <c r="B47" t="inlineStr"/>
       <c r="C47" s="3" t="inlineStr">
         <is>
           <t>Ground Wire - 12 AWG Green/Yellow</t>
@@ -1875,7 +1835,6 @@
       <c r="A48" t="n">
         <v>40</v>
       </c>
-      <c r="B48" t="inlineStr"/>
       <c r="C48" s="3" t="inlineStr">
         <is>
           <t>Fuse - 500 mA fast-blow (5x20 mm)</t>
@@ -1909,7 +1868,6 @@
       <c r="A49" t="n">
         <v>41</v>
       </c>
-      <c r="B49" t="inlineStr"/>
       <c r="C49" s="3" t="inlineStr">
         <is>
           <t>Fuse - 1 A fast-blow (5x20 mm)</t>
@@ -2566,194 +2524,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="60" customWidth="1" min="8" max="8"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Option</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Price Score (50%)</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Current Capability (20%)</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Build Quality (15%)</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Documentation / Support (10%)</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Brand / Reliability (5%)</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Total Score</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>VEVOR 3HP 120V VFD</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="n">
-        <v>9</v>
-      </c>
-      <c r="C2" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="D2" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="E2" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="F2" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="G2" s="3">
-        <f>B2*0.5+C2*0.2+D2*0.15+E2*0.1+F2*0.05</f>
-        <v/>
-      </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>Lowest cost ($70-95). Hobby-grade, limited docs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>110V 20A 3HP VFD (generic)</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="C3" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="D3" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="F3" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="G3" s="3">
-        <f>B3*0.5+C3*0.2+D3*0.15+E3*0.1+F3*0.05</f>
-        <v/>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>Best balance ($130-150). Good for 20A circuits.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Huanyang 3HP VFD (HY02D211B-T) - SELECTED</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="D4" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="E4" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="F4" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="G4" s="3">
-        <f>B4*0.5+C4*0.2+D4*0.15+E4*0.1+F4*0.05</f>
-        <v/>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>Common CNC choice ($120-200). Selected for project.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>ATO 3HP 120V VFD</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>9</v>
-      </c>
-      <c r="D5" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="E5" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="F5" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="G5" s="3">
-        <f>B5*0.5+C5*0.2+D5*0.15+E5*0.1+F5*0.05</f>
-        <v/>
-      </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>Higher quality but too expensive ($450-500).</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>